<commit_message>
June lost-deal analysis (filter 311157): finalize 20 deals with notes
Note-refined 329058 (SS), 339774 and 368136 (перестал отвечать); rebuilt
output/june_2026_result.xlsx.

https://claude.ai/code/session_01LbKBMorYebTJqJ9qvnVc6G
</commit_message>
<xml_diff>
--- a/output/june_2026_result.xlsx
+++ b/output/june_2026_result.xlsx
@@ -565,12 +565,12 @@
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>Маленькие, не окупятся</t>
+          <t>Выручка ~60М, есть своя разработка, нет маркетолога; считают дорого, «придём когда вырастем»</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>Указано SS (маленькая база) + коммент «не окупятся»</t>
+          <t>Заметки: повторно «по цене дороговаты», «придём, когда вырастем»; заметка 05.06: «выручка 60 лямов, есть разработка, нет маркетолога». Несозревший/маленький → self-service.</t>
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
@@ -630,12 +630,12 @@
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Владелец продал Паоло Пиццу (уехал в Грузию), далее не отвечает</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>Указано «не могу получить ответ», коммент пуст — нужна заметка для деталей</t>
+          <t>Заметка 03.02: «Пиццу Паоло продал давно, живу в Грузии»; дальше догон без ответа. Указано «не могу получить ответ».</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
@@ -992,17 +992,17 @@
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>Проигрыш до встречи (стек Битрикс)</t>
+          <t>После встречи основатель-ЛПР (Евгений) не вовлёкся; база email ~1000</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>Причина «Midmarket до встречи», коммент пуст — нужна заметка</t>
+          <t>Блок «Что тормозит»: ЛПР-основатель не вовлечён, маленькая база (~1000), негативный опыт email. Заметка 18.05: «ещё не пообщались».</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Owner/ЛПР veto outranks current-stack: reclassify 342605
- 342605 'собственница не согласовала' -> Руководитель заблокировал решение
- methodology: add precedence rule (step 0) — ЛПР veto wins over 'Конкурент'

https://claude.ai/code/session_01LbKBMorYebTJqJ9qvnVc6G
</commit_message>
<xml_diff>
--- a/output/june_2026_result.xlsx
+++ b/output/june_2026_result.xlsx
@@ -726,17 +726,17 @@
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Конкурент</t>
+          <t>Руководитель заблокировал решение</t>
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>Остались на своих инструментах (in-house); собственница не согласовала</t>
+          <t>Собственница не согласовала; остались на своих инструментах (in-house)</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Коммент: «собственница не согласовала, остались на своих инструментах» + стек in-house/1С</t>
+          <t>Коммент: «собственница не согласовала, остались на своих инструментах». Вето собственника (ЛПР/бюджетодержатель) приоритетнее факта текущего стека.</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">

</xml_diff>